<commit_message>
added NGS download script; modified sample naming; converted first half of notebook to .py
</commit_message>
<xml_diff>
--- a/samples.xlsx
+++ b/samples.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hadrienng/Desktop/Motif_Analysis_Automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C24D373-6F0C-534C-AFF0-AC8F59D2FB25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01404F6-07AF-B643-BFE6-F84BF4ABE52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21600" xr2:uid="{F84EA27E-2658-4342-B2DE-F04F0313C281}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="31">
   <si>
     <t>sample</t>
   </si>
@@ -108,6 +108,30 @@
   </si>
   <si>
     <t>GGCCACCGCACACCATG</t>
+  </si>
+  <si>
+    <t>replicate</t>
+  </si>
+  <si>
+    <t>A5-Psp-noPro</t>
+  </si>
+  <si>
+    <t>A6-Psp-16</t>
+  </si>
+  <si>
+    <t>A7-bt3-noPro</t>
+  </si>
+  <si>
+    <t>A8-bt3-16</t>
+  </si>
+  <si>
+    <t>A9-Rx-noPro</t>
+  </si>
+  <si>
+    <t>A10-Rx-16</t>
+  </si>
+  <si>
+    <t>A11-dict-oKW2182</t>
   </si>
 </sst>
 </file>
@@ -479,292 +503,616 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3B7966B-F68A-A947-BF58-85EDF6AEE307}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
     <col min="5" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G2">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G3">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G5">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G6">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G7">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G8">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G9">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G10">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11">
-        <v>-4</v>
+        <v>22</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="G11">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
         <v>19</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>20</v>
       </c>
-      <c r="C12" t="s">
-        <v>22</v>
-      </c>
       <c r="D12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" t="s">
         <v>21</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>0</v>
       </c>
-      <c r="F12">
-        <v>35</v>
-      </c>
       <c r="G12">
+        <v>35</v>
+      </c>
+      <c r="H12">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13">
+        <v>-4</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14">
+        <v>-4</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15">
+        <v>-4</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16">
+        <v>-4</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17">
+        <v>-4</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18">
+        <v>-4</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19">
+        <v>-4</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20">
+        <v>-4</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21">
+        <v>-4</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>2</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22">
+        <v>-4</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>35</v>
+      </c>
+      <c r="H23">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>